<commit_message>
added link to order t-shirt
added link to order t-shirt to the cast page
</commit_message>
<xml_diff>
--- a/howTo26/How2$ production.xlsx
+++ b/howTo26/How2$ production.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Seagate X/RVCOprod/website/howTo26/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB4E6FEE-4BDF-8A40-86C1-D6D13F0AA2A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94CA5CE7-6104-E848-9235-7B80D0D838CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4040" yWindow="600" windowWidth="27860" windowHeight="20600" activeTab="1" xr2:uid="{E38B6315-D279-724B-88A4-0AE2C1BF2347}"/>
+    <workbookView xWindow="10400" yWindow="600" windowWidth="27860" windowHeight="20600" activeTab="1" xr2:uid="{E38B6315-D279-724B-88A4-0AE2C1BF2347}"/>
   </bookViews>
   <sheets>
     <sheet name="Cast" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
set design, Jen videos, and tweaks to dance pages
Created updates set design jpg, added Jen videos for Pirate Dance and Cinderella Darling.
</commit_message>
<xml_diff>
--- a/howTo26/How2$ production.xlsx
+++ b/howTo26/How2$ production.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Seagate X/RVCOprod/website/howTo26/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92565AEA-86EB-F84C-B745-33A025BC2965}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AAA4280-96CB-5546-99D5-FC3FB093751A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1520" yWindow="1000" windowWidth="27860" windowHeight="20600" activeTab="1" xr2:uid="{E38B6315-D279-724B-88A4-0AE2C1BF2347}"/>
+    <workbookView xWindow="120" yWindow="600" windowWidth="27860" windowHeight="20600" activeTab="1" xr2:uid="{E38B6315-D279-724B-88A4-0AE2C1BF2347}"/>
   </bookViews>
   <sheets>
     <sheet name="Cast" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="246">
   <si>
     <t xml:space="preserve">EMERGENCY CONTACT </t>
   </si>
@@ -391,34 +391,18 @@
     <t>Down Stage Right</t>
   </si>
   <si>
-    <t>fencing and plants</t>
-  </si>
-  <si>
     <t xml:space="preserve">clear terrance </t>
   </si>
   <si>
-    <t>need couch down stage left
-skip half-wall</t>
-  </si>
-  <si>
-    <t>Back to both executive office</t>
-  </si>
-  <si>
     <t>Cinderella Darling</t>
   </si>
   <si>
     <t>Executive Office stage left</t>
   </si>
   <si>
-    <t>larger table with 7 to 8 chairs, chart easel</t>
-  </si>
-  <si>
     <t>Pirate Dance</t>
   </si>
   <si>
-    <t>chairs toppled over maybe a desk, typewriter, waste basket</t>
-  </si>
-  <si>
     <t>no change</t>
   </si>
   <si>
@@ -467,16 +451,7 @@
     <t>Closes</t>
   </si>
   <si>
-    <t>Bring in mailroom wall</t>
-  </si>
-  <si>
-    <t>need intercom</t>
-  </si>
-  <si>
     <t>see above</t>
-  </si>
-  <si>
-    <t>starts middle of pg. 23</t>
   </si>
   <si>
     <t>pg. 22 Bigley is the executive office on stage right</t>
@@ -504,10 +479,6 @@
 - Grand Old Ivy (Reprise)</t>
   </si>
   <si>
-    <t>- desk and chair for Gatch and door
-- chair &amp; desk for Miss Krumholtz</t>
-  </si>
-  <si>
     <t>Building corridor </t>
   </si>
   <si>
@@ -553,9 +524,6 @@
     <t xml:space="preserve">Stage right </t>
   </si>
   <si>
-    <t>Stage left</t>
-  </si>
-  <si>
     <t>sinks come on</t>
   </si>
   <si>
@@ -569,29 +537,6 @@
   </si>
   <si>
     <t>Office is stage right in front of Biggley's office.  Desk &amp; chair</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Traveler opens</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> but no desks  or some in front of the half-wall</t>
-    </r>
   </si>
   <si>
     <r>
@@ -651,9 +596,6 @@
     <t>Plans &amp; Systems Office</t>
   </si>
   <si>
-    <t>- desk and chair</t>
-  </si>
-  <si>
     <t>- strike mailroom stage left
 - strike outer office stage right</t>
   </si>
@@ -669,9 +611,6 @@
   <si>
     <t>Moving wall oppossite mailroom wall.
 Some guys are watching in the boardroom or not. May need an old TV.</t>
-  </si>
-  <si>
-    <t>Scrubwomen 'cleaning up'</t>
   </si>
   <si>
     <t>Book Voice Scenes</t>
@@ -894,6 +833,98 @@
   </si>
   <si>
     <t>EVERYONE</t>
+  </si>
+  <si>
+    <t>Characters</t>
+  </si>
+  <si>
+    <t>Closed</t>
+  </si>
+  <si>
+    <t>The same 4 desks as in scene 2</t>
+  </si>
+  <si>
+    <t>4 secretay desks</t>
+  </si>
+  <si>
+    <t>chairs toppled over maybe a desk, typewriter, waste basket
+Scrubwomen 'cleaning up'</t>
+  </si>
+  <si>
+    <t>Door and down stage left</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Traveler opens</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> just 4 secretary desks</t>
+    </r>
+  </si>
+  <si>
+    <t>Bring in mailroom wall; phone table on wall by the stairs stage left; table in centered of wall with wall being 3/4 feet from stage left
+Biggley table stage right</t>
+  </si>
+  <si>
+    <t>just Biggley desk and chair; need intercom</t>
+  </si>
+  <si>
+    <t>starts middle of pg. 23
+stage crew takes off Biggley desk when Twimble/Finch enter</t>
+  </si>
+  <si>
+    <t>use the other real desk</t>
+  </si>
+  <si>
+    <t>use the other real desk; down stage right</t>
+  </si>
+  <si>
+    <t>just Biggley desk and chair</t>
+  </si>
+  <si>
+    <t>same as 4.1</t>
+  </si>
+  <si>
+    <t>Same as 2/3</t>
+  </si>
+  <si>
+    <t>- desk and chair; pony wall</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- use other real desk and chair for Gatch </t>
+  </si>
+  <si>
+    <t>bar cart, fencing and plants</t>
+  </si>
+  <si>
+    <t>need couch down stage left, Biggley desk and chair stage right, door, and pony wall</t>
+  </si>
+  <si>
+    <t>no couch</t>
+  </si>
+  <si>
+    <t>larger table with 8 chairs</t>
+  </si>
+  <si>
+    <t>TV show is Stage left; business men are stage right - need 4 chairs and TV</t>
+  </si>
+  <si>
+    <t>using 4 secretary desks, 4 chairs</t>
   </si>
 </sst>
 </file>
@@ -1017,7 +1048,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1113,9 +1144,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1144,9 +1172,6 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1159,10 +1184,6 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1181,6 +1202,9 @@
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2027,7 +2051,7 @@
         <v>3</v>
       </c>
       <c r="G21" s="16" t="s">
-        <v>177</v>
+        <v>165</v>
       </c>
       <c r="H21" s="25">
         <v>19</v>
@@ -2053,7 +2077,7 @@
         <v>3</v>
       </c>
       <c r="G22" s="16" t="s">
-        <v>178</v>
+        <v>166</v>
       </c>
       <c r="H22" s="25">
         <v>20</v>
@@ -2073,7 +2097,7 @@
       <c r="E23" s="22"/>
       <c r="F23" s="9"/>
       <c r="G23" s="10" t="s">
-        <v>176</v>
+        <v>164</v>
       </c>
       <c r="H23" s="25">
         <v>21</v>
@@ -2099,7 +2123,7 @@
         <v>3</v>
       </c>
       <c r="G24" s="16" t="s">
-        <v>178</v>
+        <v>166</v>
       </c>
       <c r="H24" s="25">
         <v>22</v>
@@ -2125,7 +2149,7 @@
         <v>3</v>
       </c>
       <c r="G25" s="16" t="s">
-        <v>177</v>
+        <v>165</v>
       </c>
       <c r="H25" s="25">
         <v>23</v>
@@ -2155,7 +2179,7 @@
       <c r="A28" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="B28" s="57" t="s">
+      <c r="B28" s="53" t="s">
         <v>81</v>
       </c>
       <c r="C28" s="18">
@@ -2310,862 +2334,879 @@
   <dimension ref="A1:I44"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="4.5" style="41" customWidth="1"/>
-    <col min="2" max="2" width="5" style="41" customWidth="1"/>
-    <col min="3" max="3" width="4.83203125" style="41" customWidth="1"/>
-    <col min="4" max="4" width="14.5" style="38" customWidth="1"/>
-    <col min="5" max="5" width="7.5" style="39" customWidth="1"/>
-    <col min="6" max="6" width="26.1640625" style="40" customWidth="1"/>
-    <col min="7" max="7" width="23.5" style="41" customWidth="1"/>
-    <col min="8" max="8" width="23.5" style="42" customWidth="1"/>
-    <col min="9" max="9" width="28.1640625" style="40" customWidth="1"/>
-    <col min="10" max="16384" width="10.83203125" style="41"/>
+    <col min="1" max="1" width="4.5" style="40" customWidth="1"/>
+    <col min="2" max="2" width="5" style="40" customWidth="1"/>
+    <col min="3" max="3" width="4.83203125" style="40" customWidth="1"/>
+    <col min="4" max="4" width="14.5" style="37" customWidth="1"/>
+    <col min="5" max="5" width="7.5" style="38" customWidth="1"/>
+    <col min="6" max="6" width="26.1640625" style="39" customWidth="1"/>
+    <col min="7" max="7" width="23.5" style="40" customWidth="1"/>
+    <col min="8" max="8" width="23.5" style="39" customWidth="1"/>
+    <col min="9" max="9" width="28.1640625" style="39" customWidth="1"/>
+    <col min="10" max="16384" width="10.83203125" style="40"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" s="31" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="B1" s="33" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="C1" s="33" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="D1" s="32" t="s">
+        <v>121</v>
+      </c>
+      <c r="E1" s="33" t="s">
+        <v>125</v>
+      </c>
+      <c r="F1" s="34" t="s">
+        <v>119</v>
+      </c>
+      <c r="G1" s="31" t="s">
+        <v>120</v>
+      </c>
+      <c r="H1" s="32" t="s">
+        <v>117</v>
+      </c>
+      <c r="I1" s="32" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B2" s="36"/>
+      <c r="C2" s="36"/>
+    </row>
+    <row r="3" spans="1:9" ht="30" x14ac:dyDescent="0.2">
+      <c r="A3" s="35" t="s">
+        <v>103</v>
+      </c>
+      <c r="B3" s="42">
+        <v>1</v>
+      </c>
+      <c r="C3" s="42">
+        <v>1</v>
+      </c>
+      <c r="D3" s="43" t="s">
+        <v>122</v>
+      </c>
+      <c r="E3" s="44" t="s">
+        <v>127</v>
+      </c>
+      <c r="F3" s="39" t="s">
         <v>126</v>
       </c>
-      <c r="E1" s="33" t="s">
-        <v>130</v>
-      </c>
-      <c r="F1" s="34" t="s">
-        <v>124</v>
-      </c>
-      <c r="G1" s="31" t="s">
-        <v>125</v>
-      </c>
-      <c r="H1" s="35" t="s">
-        <v>122</v>
-      </c>
-      <c r="I1" s="34"/>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B2" s="37"/>
-      <c r="C2" s="37"/>
-    </row>
-    <row r="3" spans="1:9" ht="30" x14ac:dyDescent="0.2">
-      <c r="A3" s="36" t="s">
-        <v>103</v>
-      </c>
-      <c r="B3" s="43">
-        <v>1</v>
-      </c>
-      <c r="C3" s="43">
-        <v>1</v>
-      </c>
-      <c r="D3" s="44" t="s">
-        <v>127</v>
-      </c>
-      <c r="E3" s="45" t="s">
-        <v>132</v>
-      </c>
-      <c r="F3" s="40" t="s">
-        <v>131</v>
-      </c>
-      <c r="H3" s="46" t="s">
+      <c r="H3" s="49" t="s">
         <v>105</v>
       </c>
-      <c r="I3" s="40" t="s">
+      <c r="I3" s="39" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="4" spans="1:9" s="47" customFormat="1" ht="75" x14ac:dyDescent="0.2">
-      <c r="B4" s="43">
+    <row r="4" spans="1:9" s="45" customFormat="1" ht="75" x14ac:dyDescent="0.2">
+      <c r="B4" s="42">
         <f>B3+1</f>
         <v>2</v>
       </c>
-      <c r="C4" s="43">
+      <c r="C4" s="42">
         <v>2</v>
       </c>
-      <c r="D4" s="44" t="s">
+      <c r="D4" s="43" t="s">
+        <v>123</v>
+      </c>
+      <c r="E4" s="46" t="s">
         <v>128</v>
       </c>
-      <c r="E4" s="48" t="s">
-        <v>133</v>
-      </c>
-      <c r="F4" s="40" t="s">
-        <v>170</v>
-      </c>
-      <c r="H4" s="49" t="s">
-        <v>171</v>
-      </c>
-      <c r="I4" s="40" t="s">
-        <v>191</v>
+      <c r="F4" s="39" t="s">
+        <v>229</v>
+      </c>
+      <c r="H4" s="47" t="s">
+        <v>160</v>
+      </c>
+      <c r="I4" s="39" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="60" x14ac:dyDescent="0.2">
-      <c r="B5" s="43">
+      <c r="B5" s="42">
         <f t="shared" ref="B5:B24" si="0">B4+1</f>
         <v>3</v>
       </c>
-      <c r="C5" s="43">
+      <c r="C5" s="42">
         <v>13</v>
       </c>
-      <c r="D5" s="44" t="s">
-        <v>129</v>
-      </c>
-      <c r="E5" s="45" t="s">
-        <v>134</v>
-      </c>
-      <c r="H5" s="46" t="s">
-        <v>121</v>
-      </c>
-      <c r="I5" s="40" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="30" x14ac:dyDescent="0.2">
-      <c r="B6" s="43">
+      <c r="D5" s="43" t="s">
+        <v>124</v>
+      </c>
+      <c r="E5" s="44" t="s">
+        <v>224</v>
+      </c>
+      <c r="H5" s="49" t="s">
+        <v>116</v>
+      </c>
+      <c r="I5" s="39" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="75" x14ac:dyDescent="0.2">
+      <c r="B6" s="42">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C6" s="43">
+      <c r="C6" s="42">
         <v>22</v>
       </c>
-      <c r="D6" s="44" t="s">
+      <c r="D6" s="43" t="s">
         <v>107</v>
       </c>
-      <c r="E6" s="45" t="s">
-        <v>134</v>
-      </c>
-      <c r="F6" s="40" t="s">
-        <v>144</v>
-      </c>
-      <c r="G6" s="42" t="s">
+      <c r="E6" s="44" t="s">
+        <v>129</v>
+      </c>
+      <c r="F6" s="39" t="s">
         <v>136</v>
       </c>
-      <c r="I6" s="40" t="s">
-        <v>192</v>
+      <c r="G6" s="41" t="s">
+        <v>230</v>
+      </c>
+      <c r="I6" s="39" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="30" x14ac:dyDescent="0.2">
-      <c r="B7" s="43">
+      <c r="B7" s="42">
         <v>4.0999999999999996</v>
       </c>
-      <c r="C7" s="43">
+      <c r="C7" s="42">
         <v>22</v>
       </c>
-      <c r="D7" s="50" t="s">
+      <c r="D7" s="48" t="s">
         <v>106</v>
       </c>
-      <c r="E7" s="45" t="s">
-        <v>134</v>
-      </c>
-      <c r="F7" s="40" t="s">
-        <v>140</v>
-      </c>
-      <c r="G7" s="42" t="s">
-        <v>137</v>
-      </c>
-      <c r="I7" s="40" t="s">
-        <v>193</v>
+      <c r="E7" s="44" t="s">
+        <v>127</v>
+      </c>
+      <c r="F7" s="39" t="s">
+        <v>132</v>
+      </c>
+      <c r="G7" s="41" t="s">
+        <v>231</v>
+      </c>
+      <c r="I7" s="39" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="60" x14ac:dyDescent="0.2">
-      <c r="B8" s="43">
+      <c r="B8" s="42">
         <v>4.2</v>
       </c>
-      <c r="C8" s="43">
+      <c r="C8" s="42">
         <v>23</v>
       </c>
-      <c r="D8" s="50" t="s">
+      <c r="D8" s="48" t="s">
         <v>107</v>
       </c>
-      <c r="E8" s="45" t="s">
-        <v>134</v>
-      </c>
-      <c r="F8" s="40" t="s">
-        <v>138</v>
-      </c>
-      <c r="G8" s="42" t="s">
-        <v>139</v>
-      </c>
-      <c r="H8" s="51" t="s">
-        <v>194</v>
-      </c>
-      <c r="I8" s="40" t="s">
-        <v>195</v>
+      <c r="E8" s="44" t="s">
+        <v>127</v>
+      </c>
+      <c r="F8" s="39" t="s">
+        <v>131</v>
+      </c>
+      <c r="G8" s="41" t="s">
+        <v>232</v>
+      </c>
+      <c r="H8" s="47" t="s">
+        <v>181</v>
+      </c>
+      <c r="I8" s="39" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="45" x14ac:dyDescent="0.2">
-      <c r="B9" s="43">
+      <c r="B9" s="42">
         <v>4.2</v>
       </c>
-      <c r="C9" s="43">
+      <c r="C9" s="42">
         <v>33</v>
       </c>
-      <c r="D9" s="44" t="s">
+      <c r="D9" s="43" t="s">
+        <v>124</v>
+      </c>
+      <c r="E9" s="44" t="s">
         <v>129</v>
       </c>
-      <c r="E9" s="45" t="s">
-        <v>134</v>
-      </c>
-      <c r="F9" s="40" t="s">
-        <v>169</v>
-      </c>
-      <c r="G9" s="54" t="s">
-        <v>175</v>
-      </c>
-      <c r="H9" s="51" t="s">
-        <v>196</v>
-      </c>
-      <c r="I9" s="40" t="s">
-        <v>198</v>
+      <c r="F9" s="39" t="s">
+        <v>159</v>
+      </c>
+      <c r="G9" s="50" t="s">
+        <v>163</v>
+      </c>
+      <c r="H9" s="47" t="s">
+        <v>183</v>
+      </c>
+      <c r="I9" s="39" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="15" x14ac:dyDescent="0.2">
-      <c r="B10" s="43">
+      <c r="B10" s="42">
         <v>4.2</v>
       </c>
-      <c r="C10" s="43"/>
-      <c r="D10" s="44"/>
-      <c r="E10" s="45"/>
-      <c r="G10" s="54"/>
-      <c r="H10" s="51" t="s">
-        <v>197</v>
-      </c>
-      <c r="I10" s="40" t="s">
-        <v>199</v>
+      <c r="C10" s="42"/>
+      <c r="D10" s="43"/>
+      <c r="E10" s="44"/>
+      <c r="G10" s="50"/>
+      <c r="H10" s="47" t="s">
+        <v>184</v>
+      </c>
+      <c r="I10" s="39" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="15" x14ac:dyDescent="0.2">
-      <c r="B11" s="43">
+      <c r="B11" s="42">
         <f>B6+1</f>
         <v>5</v>
       </c>
-      <c r="C11" s="43">
+      <c r="C11" s="42">
         <v>38</v>
       </c>
-      <c r="D11" s="44" t="s">
-        <v>141</v>
-      </c>
-      <c r="E11" s="45" t="s">
+      <c r="D11" s="43" t="s">
+        <v>133</v>
+      </c>
+      <c r="E11" s="44" t="s">
+        <v>129</v>
+      </c>
+      <c r="F11" s="39" t="s">
+        <v>236</v>
+      </c>
+      <c r="G11" s="40" t="s">
+        <v>235</v>
+      </c>
+      <c r="I11" s="39" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="30" x14ac:dyDescent="0.2">
+      <c r="B12" s="42">
+        <v>6.1</v>
+      </c>
+      <c r="C12" s="42">
+        <v>40</v>
+      </c>
+      <c r="D12" s="43" t="s">
         <v>134</v>
       </c>
-      <c r="I11" s="40" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="30" x14ac:dyDescent="0.2">
-      <c r="B12" s="43">
-        <v>6.1</v>
-      </c>
-      <c r="C12" s="43">
-        <v>40</v>
-      </c>
-      <c r="D12" s="44" t="s">
-        <v>142</v>
-      </c>
-      <c r="E12" s="45" t="s">
-        <v>134</v>
-      </c>
-      <c r="F12" s="40" t="s">
-        <v>108</v>
-      </c>
-      <c r="G12" s="54"/>
-      <c r="H12" s="46"/>
-      <c r="I12" s="40" t="s">
-        <v>201</v>
+      <c r="E12" s="44" t="s">
+        <v>129</v>
+      </c>
+      <c r="F12" s="39" t="s">
+        <v>237</v>
+      </c>
+      <c r="G12" s="50" t="s">
+        <v>225</v>
+      </c>
+      <c r="H12" s="49"/>
+      <c r="I12" s="39" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="15" x14ac:dyDescent="0.2">
-      <c r="B13" s="43">
+      <c r="B13" s="42">
         <v>6.2</v>
       </c>
-      <c r="C13" s="43">
+      <c r="C13" s="42">
         <v>42</v>
       </c>
-      <c r="D13" s="44"/>
-      <c r="E13" s="45"/>
-      <c r="G13" s="54"/>
-      <c r="H13" s="51" t="s">
-        <v>200</v>
-      </c>
-      <c r="I13" s="40" t="s">
-        <v>202</v>
+      <c r="D13" s="43"/>
+      <c r="E13" s="44"/>
+      <c r="G13" s="50"/>
+      <c r="H13" s="47" t="s">
+        <v>187</v>
+      </c>
+      <c r="I13" s="39" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="45" x14ac:dyDescent="0.2">
-      <c r="B14" s="43">
+      <c r="B14" s="42">
         <f>B12+1</f>
         <v>7.1</v>
       </c>
-      <c r="C14" s="43">
+      <c r="C14" s="42">
         <v>45</v>
       </c>
-      <c r="D14" s="44" t="s">
-        <v>146</v>
-      </c>
-      <c r="E14" s="45" t="s">
-        <v>134</v>
-      </c>
-      <c r="F14" s="40" t="s">
+      <c r="D14" s="43" t="s">
+        <v>138</v>
+      </c>
+      <c r="E14" s="44" t="s">
+        <v>129</v>
+      </c>
+      <c r="F14" s="39" t="s">
         <v>108</v>
       </c>
-      <c r="H14" s="41"/>
-      <c r="I14" s="40" t="s">
-        <v>203</v>
+      <c r="H14" s="45"/>
+      <c r="I14" s="39" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="30" x14ac:dyDescent="0.2">
-      <c r="B15" s="43">
+      <c r="B15" s="42">
         <v>7.2</v>
       </c>
-      <c r="C15" s="43">
+      <c r="C15" s="42">
         <v>49</v>
       </c>
-      <c r="D15" s="44"/>
-      <c r="E15" s="45"/>
-      <c r="H15" s="51" t="s">
-        <v>204</v>
-      </c>
-      <c r="I15" s="40" t="s">
-        <v>206</v>
+      <c r="D15" s="43"/>
+      <c r="E15" s="44"/>
+      <c r="H15" s="47" t="s">
+        <v>191</v>
+      </c>
+      <c r="I15" s="39" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="15" x14ac:dyDescent="0.2">
-      <c r="B16" s="43">
+      <c r="B16" s="42">
         <v>7.2</v>
       </c>
-      <c r="C16" s="43">
+      <c r="C16" s="42">
         <v>55</v>
       </c>
-      <c r="D16" s="44"/>
-      <c r="E16" s="45"/>
-      <c r="H16" s="51" t="s">
-        <v>205</v>
-      </c>
-      <c r="I16" s="40" t="s">
-        <v>207</v>
+      <c r="D16" s="43"/>
+      <c r="E16" s="44"/>
+      <c r="H16" s="47" t="s">
+        <v>192</v>
+      </c>
+      <c r="I16" s="39" t="s">
+        <v>194</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="30" x14ac:dyDescent="0.2">
-      <c r="B17" s="43">
+      <c r="B17" s="42">
         <f>B14+1</f>
         <v>8.1</v>
       </c>
-      <c r="C17" s="43">
+      <c r="C17" s="42">
         <v>56</v>
       </c>
-      <c r="D17" s="44" t="s">
+      <c r="D17" s="43" t="s">
+        <v>124</v>
+      </c>
+      <c r="E17" s="44" t="s">
         <v>129</v>
       </c>
-      <c r="E17" s="45" t="s">
-        <v>134</v>
-      </c>
-      <c r="F17" s="40" t="s">
-        <v>108</v>
-      </c>
-      <c r="H17" s="51" t="s">
-        <v>147</v>
-      </c>
-      <c r="I17" s="40" t="s">
-        <v>208</v>
+      <c r="F17" s="39" t="s">
+        <v>234</v>
+      </c>
+      <c r="H17" s="47" t="s">
+        <v>139</v>
+      </c>
+      <c r="I17" s="39" t="s">
+        <v>195</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="15" x14ac:dyDescent="0.2">
-      <c r="B18" s="43">
+      <c r="B18" s="42">
         <f t="shared" si="0"/>
         <v>9.1</v>
       </c>
-      <c r="C18" s="43">
+      <c r="C18" s="42">
         <v>64</v>
       </c>
-      <c r="D18" s="44" t="s">
-        <v>145</v>
-      </c>
-      <c r="E18" s="45" t="s">
-        <v>134</v>
-      </c>
-      <c r="F18" s="40" t="s">
+      <c r="D18" s="43" t="s">
+        <v>137</v>
+      </c>
+      <c r="E18" s="44" t="s">
+        <v>129</v>
+      </c>
+      <c r="F18" s="39" t="s">
         <v>109</v>
       </c>
-      <c r="G18" s="56" t="s">
-        <v>174</v>
-      </c>
-      <c r="I18" s="40" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" ht="45" x14ac:dyDescent="0.2">
-      <c r="B19" s="43">
+      <c r="G18" s="52" t="s">
+        <v>238</v>
+      </c>
+      <c r="I18" s="39" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="30" x14ac:dyDescent="0.2">
+      <c r="B19" s="42">
         <f t="shared" si="0"/>
         <v>10.1</v>
       </c>
-      <c r="C19" s="43">
+      <c r="C19" s="42">
         <v>68</v>
       </c>
-      <c r="D19" s="44" t="s">
-        <v>173</v>
-      </c>
-      <c r="E19" s="45" t="s">
-        <v>134</v>
-      </c>
-      <c r="F19" s="40" t="s">
+      <c r="D19" s="43" t="s">
+        <v>162</v>
+      </c>
+      <c r="E19" s="44" t="s">
+        <v>129</v>
+      </c>
+      <c r="F19" s="39" t="s">
         <v>110</v>
       </c>
-      <c r="G19" s="55" t="s">
-        <v>148</v>
-      </c>
-      <c r="I19" s="40" t="s">
-        <v>210</v>
+      <c r="G19" s="51" t="s">
+        <v>239</v>
+      </c>
+      <c r="I19" s="39" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="30" x14ac:dyDescent="0.2">
-      <c r="B20" s="43">
+      <c r="B20" s="42">
         <f t="shared" si="0"/>
         <v>11.1</v>
       </c>
-      <c r="C20" s="43">
+      <c r="C20" s="42">
         <v>69</v>
       </c>
-      <c r="D20" s="44" t="s">
-        <v>149</v>
-      </c>
-      <c r="E20" s="48" t="s">
-        <v>135</v>
-      </c>
-      <c r="F20" s="40" t="s">
+      <c r="D20" s="43" t="s">
+        <v>140</v>
+      </c>
+      <c r="E20" s="46" t="s">
+        <v>130</v>
+      </c>
+      <c r="F20" s="39" t="s">
         <v>104</v>
       </c>
-      <c r="G20" s="38" t="s">
-        <v>152</v>
-      </c>
-      <c r="H20" s="46"/>
-      <c r="I20" s="40" t="s">
-        <v>211</v>
+      <c r="G20" s="37" t="s">
+        <v>143</v>
+      </c>
+      <c r="H20" s="49"/>
+      <c r="I20" s="39" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="15" x14ac:dyDescent="0.2">
-      <c r="B21" s="43"/>
-      <c r="C21" s="43"/>
-      <c r="D21" s="44"/>
-      <c r="E21" s="48"/>
-      <c r="G21" s="38"/>
-      <c r="H21" s="51" t="s">
-        <v>212</v>
-      </c>
-      <c r="I21" s="40" t="s">
-        <v>213</v>
+      <c r="B21" s="42"/>
+      <c r="C21" s="42"/>
+      <c r="D21" s="43"/>
+      <c r="E21" s="46"/>
+      <c r="G21" s="37"/>
+      <c r="H21" s="47" t="s">
+        <v>199</v>
+      </c>
+      <c r="I21" s="39" t="s">
+        <v>200</v>
       </c>
     </row>
     <row r="22" spans="1:9" ht="45" x14ac:dyDescent="0.2">
-      <c r="B22" s="43">
+      <c r="B22" s="42">
         <f>B20+1</f>
         <v>12.1</v>
       </c>
-      <c r="C22" s="43">
+      <c r="C22" s="42">
         <v>72</v>
       </c>
-      <c r="D22" s="44" t="s">
-        <v>150</v>
-      </c>
-      <c r="E22" s="48" t="s">
-        <v>133</v>
-      </c>
-      <c r="F22" s="41" t="s">
-        <v>111</v>
-      </c>
-      <c r="H22" s="54" t="s">
-        <v>214</v>
-      </c>
-      <c r="I22" s="40" t="s">
-        <v>215</v>
+      <c r="D22" s="43" t="s">
+        <v>141</v>
+      </c>
+      <c r="E22" s="46" t="s">
+        <v>128</v>
+      </c>
+      <c r="F22" s="45" t="s">
+        <v>240</v>
+      </c>
+      <c r="H22" s="51" t="s">
+        <v>201</v>
+      </c>
+      <c r="I22" s="39" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="23" spans="1:9" ht="15" x14ac:dyDescent="0.2">
-      <c r="B23" s="43">
+      <c r="B23" s="42">
         <f t="shared" si="0"/>
         <v>13.1</v>
       </c>
-      <c r="C23" s="43">
+      <c r="C23" s="42">
         <v>76</v>
       </c>
-      <c r="D23" s="44" t="s">
-        <v>146</v>
-      </c>
-      <c r="E23" s="45" t="s">
-        <v>134</v>
-      </c>
-      <c r="G23" s="41" t="s">
-        <v>112</v>
-      </c>
-      <c r="I23" s="40" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" ht="30" x14ac:dyDescent="0.2">
-      <c r="B24" s="43">
+      <c r="D23" s="43" t="s">
+        <v>138</v>
+      </c>
+      <c r="E23" s="44" t="s">
+        <v>129</v>
+      </c>
+      <c r="G23" s="40" t="s">
+        <v>111</v>
+      </c>
+      <c r="I23" s="39" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="45" x14ac:dyDescent="0.2">
+      <c r="B24" s="42">
         <f t="shared" si="0"/>
         <v>14.1</v>
       </c>
-      <c r="C24" s="43">
+      <c r="C24" s="42">
         <v>79</v>
       </c>
-      <c r="D24" s="44" t="s">
-        <v>151</v>
-      </c>
-      <c r="E24" s="45" t="s">
-        <v>134</v>
-      </c>
-      <c r="F24" s="38" t="s">
-        <v>113</v>
-      </c>
-      <c r="H24" s="41"/>
-      <c r="I24" s="40" t="s">
-        <v>217</v>
+      <c r="D24" s="43" t="s">
+        <v>142</v>
+      </c>
+      <c r="E24" s="44" t="s">
+        <v>129</v>
+      </c>
+      <c r="F24" s="37" t="s">
+        <v>241</v>
+      </c>
+      <c r="H24" s="45"/>
+      <c r="I24" s="39" t="s">
+        <v>204</v>
       </c>
     </row>
     <row r="25" spans="1:9" ht="30" x14ac:dyDescent="0.2">
-      <c r="B25" s="43">
+      <c r="B25" s="42">
         <v>14.2</v>
       </c>
-      <c r="C25" s="43">
+      <c r="C25" s="42">
         <v>81</v>
       </c>
-      <c r="D25" s="44"/>
-      <c r="E25" s="45"/>
-      <c r="F25" s="38"/>
-      <c r="H25" s="51" t="s">
-        <v>221</v>
-      </c>
-      <c r="I25" s="40" t="s">
-        <v>218</v>
+      <c r="D25" s="43"/>
+      <c r="E25" s="44"/>
+      <c r="F25" s="37"/>
+      <c r="H25" s="47" t="s">
+        <v>208</v>
+      </c>
+      <c r="I25" s="39" t="s">
+        <v>205</v>
       </c>
     </row>
     <row r="26" spans="1:9" ht="15" x14ac:dyDescent="0.2">
-      <c r="B26" s="43">
+      <c r="B26" s="42">
         <v>14.3</v>
       </c>
-      <c r="C26" s="43">
+      <c r="C26" s="42">
         <v>87</v>
       </c>
-      <c r="D26" s="44"/>
-      <c r="E26" s="45"/>
-      <c r="F26" s="38"/>
-      <c r="H26" s="51" t="s">
-        <v>219</v>
-      </c>
-      <c r="I26" s="40" t="s">
-        <v>220</v>
+      <c r="D26" s="43"/>
+      <c r="E26" s="44"/>
+      <c r="F26" s="37"/>
+      <c r="H26" s="47" t="s">
+        <v>206</v>
+      </c>
+      <c r="I26" s="39" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="27" spans="1:9" ht="15" x14ac:dyDescent="0.2">
-      <c r="B27" s="43">
+      <c r="B27" s="42">
         <v>14.4</v>
       </c>
-      <c r="C27" s="39">
+      <c r="C27" s="38">
         <v>91</v>
       </c>
-      <c r="D27" s="40"/>
-      <c r="E27" s="43"/>
-      <c r="H27" s="54" t="s">
-        <v>222</v>
-      </c>
-      <c r="I27" s="40" t="s">
-        <v>223</v>
+      <c r="D27" s="39"/>
+      <c r="E27" s="42"/>
+      <c r="H27" s="51" t="s">
+        <v>209</v>
+      </c>
+      <c r="I27" s="39" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="28" spans="1:9" ht="45" x14ac:dyDescent="0.2">
-      <c r="A28" s="36" t="s">
-        <v>153</v>
-      </c>
-      <c r="B28" s="43">
+      <c r="A28" s="35" t="s">
+        <v>144</v>
+      </c>
+      <c r="B28" s="42">
         <v>1</v>
       </c>
-      <c r="C28" s="43">
+      <c r="C28" s="42">
         <v>93</v>
       </c>
-      <c r="D28" s="44" t="s">
-        <v>129</v>
-      </c>
-      <c r="E28" s="48" t="s">
-        <v>133</v>
-      </c>
-      <c r="F28" s="40" t="s">
-        <v>114</v>
-      </c>
-      <c r="H28" s="52" t="s">
-        <v>115</v>
-      </c>
-      <c r="I28" s="40" t="s">
-        <v>224</v>
+      <c r="D28" s="43" t="s">
+        <v>124</v>
+      </c>
+      <c r="E28" s="46" t="s">
+        <v>128</v>
+      </c>
+      <c r="F28" s="39" t="s">
+        <v>226</v>
+      </c>
+      <c r="H28" s="56" t="s">
+        <v>112</v>
+      </c>
+      <c r="I28" s="39" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="29" spans="1:9" ht="30" x14ac:dyDescent="0.2">
-      <c r="B29" s="43">
+      <c r="B29" s="42">
         <f t="shared" ref="B29:B35" si="1">B28+1</f>
         <v>2</v>
       </c>
-      <c r="C29" s="43">
+      <c r="C29" s="42">
         <v>99</v>
       </c>
-      <c r="D29" s="44" t="s">
-        <v>154</v>
-      </c>
-      <c r="E29" s="45" t="s">
-        <v>134</v>
-      </c>
-      <c r="F29" s="40" t="s">
-        <v>116</v>
-      </c>
-      <c r="H29" s="46" t="s">
-        <v>156</v>
-      </c>
-      <c r="I29" s="40" t="s">
-        <v>225</v>
+      <c r="D29" s="43" t="s">
+        <v>145</v>
+      </c>
+      <c r="E29" s="44" t="s">
+        <v>129</v>
+      </c>
+      <c r="F29" s="39" t="s">
+        <v>113</v>
+      </c>
+      <c r="G29" s="45" t="s">
+        <v>233</v>
+      </c>
+      <c r="H29" s="49" t="s">
+        <v>147</v>
+      </c>
+      <c r="I29" s="39" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="30" spans="1:9" ht="15" x14ac:dyDescent="0.2">
-      <c r="B30" s="43">
+      <c r="B30" s="42">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="C30" s="43">
+      <c r="C30" s="42">
         <v>105</v>
       </c>
-      <c r="D30" s="44" t="s">
-        <v>155</v>
-      </c>
-      <c r="E30" s="45" t="s">
-        <v>134</v>
-      </c>
-      <c r="H30" s="46" t="s">
-        <v>158</v>
-      </c>
-      <c r="I30" s="40" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" s="47" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="B31" s="43">
+      <c r="D30" s="43" t="s">
+        <v>146</v>
+      </c>
+      <c r="E30" s="44" t="s">
+        <v>129</v>
+      </c>
+      <c r="G30" s="40" t="s">
+        <v>242</v>
+      </c>
+      <c r="H30" s="49" t="s">
+        <v>149</v>
+      </c>
+      <c r="I30" s="39" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" s="45" customFormat="1" ht="30" x14ac:dyDescent="0.2">
+      <c r="B31" s="42">
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="C31" s="43">
+      <c r="C31" s="42">
         <v>111</v>
       </c>
-      <c r="D31" s="44" t="s">
-        <v>157</v>
-      </c>
-      <c r="E31" s="48" t="s">
-        <v>135</v>
-      </c>
-      <c r="F31" s="40"/>
-      <c r="G31" s="47" t="s">
-        <v>165</v>
-      </c>
-      <c r="H31" s="53" t="s">
-        <v>159</v>
-      </c>
-      <c r="I31" s="40" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" s="47" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="B32" s="43">
+      <c r="D31" s="43" t="s">
+        <v>148</v>
+      </c>
+      <c r="E31" s="46" t="s">
+        <v>130</v>
+      </c>
+      <c r="F31" s="39"/>
+      <c r="G31" s="45" t="s">
+        <v>155</v>
+      </c>
+      <c r="H31" s="49" t="s">
+        <v>150</v>
+      </c>
+      <c r="I31" s="39" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" s="45" customFormat="1" ht="45" x14ac:dyDescent="0.2">
+      <c r="B32" s="42">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="C32" s="43">
+      <c r="C32" s="42">
         <v>115</v>
       </c>
-      <c r="D32" s="44" t="s">
-        <v>160</v>
-      </c>
-      <c r="E32" s="45" t="s">
-        <v>132</v>
-      </c>
-      <c r="F32" s="40" t="s">
-        <v>163</v>
-      </c>
-      <c r="G32" s="40" t="s">
-        <v>117</v>
-      </c>
-      <c r="H32" s="40"/>
-      <c r="I32" s="40" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="33" spans="2:9" s="47" customFormat="1" ht="75" x14ac:dyDescent="0.2">
-      <c r="B33" s="43">
+      <c r="D32" s="43" t="s">
+        <v>151</v>
+      </c>
+      <c r="E32" s="44" t="s">
+        <v>127</v>
+      </c>
+      <c r="F32" s="39" t="s">
+        <v>154</v>
+      </c>
+      <c r="G32" s="39" t="s">
+        <v>243</v>
+      </c>
+      <c r="H32" s="39"/>
+      <c r="I32" s="39" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="33" spans="2:9" s="45" customFormat="1" ht="75" x14ac:dyDescent="0.2">
+      <c r="B33" s="42">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="C33" s="43">
+      <c r="C33" s="42">
         <v>125</v>
       </c>
-      <c r="D33" s="44" t="s">
-        <v>161</v>
-      </c>
-      <c r="E33" s="45" t="s">
-        <v>132</v>
-      </c>
-      <c r="F33" s="40" t="s">
-        <v>164</v>
-      </c>
-      <c r="G33" s="40" t="s">
-        <v>179</v>
-      </c>
-      <c r="H33" s="40" t="s">
-        <v>118</v>
-      </c>
-      <c r="I33" s="40" t="s">
-        <v>229</v>
+      <c r="D33" s="43" t="s">
+        <v>152</v>
+      </c>
+      <c r="E33" s="44" t="s">
+        <v>127</v>
+      </c>
+      <c r="F33" s="39" t="s">
+        <v>244</v>
+      </c>
+      <c r="G33" s="39" t="s">
+        <v>167</v>
+      </c>
+      <c r="H33" s="39" t="s">
+        <v>114</v>
+      </c>
+      <c r="I33" s="39" t="s">
+        <v>216</v>
       </c>
     </row>
     <row r="34" spans="2:9" ht="45" x14ac:dyDescent="0.2">
-      <c r="B34" s="43">
+      <c r="B34" s="42">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="C34" s="43">
+      <c r="C34" s="42">
         <v>128</v>
       </c>
-      <c r="D34" s="44" t="s">
-        <v>162</v>
-      </c>
-      <c r="E34" s="48" t="s">
-        <v>133</v>
-      </c>
-      <c r="G34" s="42" t="s">
-        <v>119</v>
-      </c>
-      <c r="H34" s="46" t="s">
-        <v>166</v>
-      </c>
-      <c r="I34" s="40" t="s">
-        <v>230</v>
+      <c r="D34" s="43" t="s">
+        <v>153</v>
+      </c>
+      <c r="E34" s="46" t="s">
+        <v>128</v>
+      </c>
+      <c r="F34" s="39" t="s">
+        <v>245</v>
+      </c>
+      <c r="G34" s="41" t="s">
+        <v>227</v>
+      </c>
+      <c r="H34" s="49" t="s">
+        <v>156</v>
+      </c>
+      <c r="I34" s="39" t="s">
+        <v>217</v>
       </c>
     </row>
     <row r="35" spans="2:9" ht="15" x14ac:dyDescent="0.2">
-      <c r="B35" s="43">
+      <c r="B35" s="42">
         <f t="shared" si="1"/>
         <v>8</v>
       </c>
-      <c r="C35" s="43">
+      <c r="C35" s="42">
         <v>133</v>
       </c>
-      <c r="D35" s="44" t="s">
+      <c r="D35" s="43"/>
+      <c r="E35" s="44" t="s">
+        <v>129</v>
+      </c>
+      <c r="F35" s="39" t="s">
+        <v>228</v>
+      </c>
+      <c r="I35" s="39" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="36" spans="2:9" ht="45" x14ac:dyDescent="0.2">
+      <c r="B36" s="42">
+        <v>9.1</v>
+      </c>
+      <c r="C36" s="42">
+        <v>134</v>
+      </c>
+      <c r="D36" s="43" t="s">
         <v>146</v>
       </c>
-      <c r="E35" s="45" t="s">
-        <v>134</v>
-      </c>
-      <c r="G35" s="41" t="s">
-        <v>180</v>
-      </c>
-      <c r="I35" s="40" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="36" spans="2:9" ht="45" x14ac:dyDescent="0.2">
-      <c r="B36" s="43">
-        <v>9.1</v>
-      </c>
-      <c r="C36" s="43">
-        <v>134</v>
-      </c>
-      <c r="D36" s="44" t="s">
-        <v>155</v>
-      </c>
-      <c r="E36" s="45" t="s">
-        <v>134</v>
-      </c>
-      <c r="F36" s="40" t="s">
-        <v>120</v>
-      </c>
-      <c r="H36" s="41"/>
-      <c r="I36" s="40" t="s">
-        <v>233</v>
+      <c r="E36" s="44" t="s">
+        <v>129</v>
+      </c>
+      <c r="F36" s="39" t="s">
+        <v>115</v>
+      </c>
+      <c r="H36" s="45"/>
+      <c r="I36" s="39" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="37" spans="2:9" ht="30" x14ac:dyDescent="0.2">
-      <c r="B37" s="43">
+      <c r="B37" s="42">
         <v>9.1999999999999993</v>
       </c>
-      <c r="C37" s="43">
+      <c r="C37" s="42">
         <v>139</v>
       </c>
-      <c r="D37" s="44" t="s">
-        <v>168</v>
-      </c>
-      <c r="E37" s="45" t="s">
-        <v>134</v>
-      </c>
-      <c r="H37" s="46" t="s">
-        <v>167</v>
-      </c>
-      <c r="I37" s="40" t="s">
-        <v>232</v>
+      <c r="D37" s="43" t="s">
+        <v>158</v>
+      </c>
+      <c r="E37" s="44" t="s">
+        <v>129</v>
+      </c>
+      <c r="H37" s="49" t="s">
+        <v>157</v>
+      </c>
+      <c r="I37" s="39" t="s">
+        <v>219</v>
       </c>
     </row>
     <row r="38" spans="2:9" ht="15" x14ac:dyDescent="0.2">
-      <c r="B38" s="43" t="s">
-        <v>234</v>
-      </c>
-      <c r="C38" s="43">
+      <c r="B38" s="42" t="s">
+        <v>221</v>
+      </c>
+      <c r="C38" s="42">
         <v>143</v>
       </c>
-      <c r="D38" s="44"/>
-      <c r="E38" s="45"/>
-      <c r="H38" s="46"/>
-      <c r="I38" s="40" t="s">
-        <v>235</v>
+      <c r="D38" s="43"/>
+      <c r="E38" s="44"/>
+      <c r="H38" s="49"/>
+      <c r="I38" s="39" t="s">
+        <v>222</v>
       </c>
     </row>
     <row r="39" spans="2:9" ht="30" x14ac:dyDescent="0.2">
-      <c r="B39" s="43">
+      <c r="B39" s="42">
         <f>B36+1</f>
         <v>10.1</v>
       </c>
-      <c r="C39" s="43">
+      <c r="C39" s="42">
         <v>143</v>
       </c>
-      <c r="D39" s="44" t="s">
+      <c r="D39" s="43" t="s">
+        <v>124</v>
+      </c>
+      <c r="E39" s="44" t="s">
         <v>129</v>
       </c>
-      <c r="E39" s="45" t="s">
-        <v>134</v>
-      </c>
-      <c r="F39" s="40" t="s">
-        <v>120</v>
-      </c>
-      <c r="H39" s="54" t="s">
-        <v>172</v>
-      </c>
-      <c r="I39" s="40" t="s">
-        <v>235</v>
+      <c r="F39" s="39" t="s">
+        <v>115</v>
+      </c>
+      <c r="H39" s="51" t="s">
+        <v>161</v>
+      </c>
+      <c r="I39" s="39" t="s">
+        <v>222</v>
       </c>
     </row>
     <row r="40" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B40" s="43"/>
-      <c r="C40" s="43"/>
-      <c r="D40" s="44"/>
-      <c r="E40" s="45"/>
+      <c r="B40" s="42"/>
+      <c r="C40" s="42"/>
+      <c r="D40" s="43"/>
+      <c r="E40" s="44"/>
     </row>
     <row r="41" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="D41" s="40"/>
-      <c r="E41" s="43"/>
+      <c r="D41" s="39"/>
+      <c r="E41" s="42"/>
     </row>
     <row r="42" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="D42" s="44"/>
-      <c r="E42" s="45"/>
+      <c r="D42" s="43"/>
+      <c r="E42" s="44"/>
     </row>
     <row r="43" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="D43" s="44"/>
-      <c r="E43" s="45"/>
+      <c r="D43" s="43"/>
+      <c r="E43" s="44"/>
     </row>
     <row r="44" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="D44" s="44"/>
-      <c r="E44" s="45"/>
+      <c r="D44" s="43"/>
+      <c r="E44" s="44"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3184,13 +3225,13 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" s="59" t="s">
-        <v>181</v>
+      <c r="A2" s="55" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B4" s="27" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="195" customHeight="1" x14ac:dyDescent="0.2">
@@ -3200,67 +3241,67 @@
       <c r="B5" s="27">
         <v>1</v>
       </c>
-      <c r="C5" s="58" t="s">
-        <v>182</v>
+      <c r="C5" s="54" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="65" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="27">
         <v>2</v>
       </c>
-      <c r="C6" s="58" t="s">
-        <v>183</v>
+      <c r="C6" s="54" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="77" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="27">
         <v>3</v>
       </c>
-      <c r="C7" s="58" t="s">
-        <v>184</v>
+      <c r="C7" s="54" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="27">
         <v>5</v>
       </c>
-      <c r="C8" s="58" t="s">
-        <v>185</v>
+      <c r="C8" s="54" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="163" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="27">
         <v>9</v>
       </c>
-      <c r="C9" s="58" t="s">
-        <v>186</v>
+      <c r="C9" s="54" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="102" x14ac:dyDescent="0.2">
       <c r="A10" s="26" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="B10" s="27">
         <v>2</v>
       </c>
-      <c r="C10" s="58" t="s">
-        <v>187</v>
+      <c r="C10" s="54" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B11" s="27">
         <v>5</v>
       </c>
-      <c r="C11" s="58" t="s">
-        <v>188</v>
+      <c r="C11" s="54" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="85" x14ac:dyDescent="0.2">
       <c r="B12" s="27">
         <v>7</v>
       </c>
-      <c r="C12" s="58" t="s">
-        <v>189</v>
+      <c r="C12" s="54" t="s">
+        <v>176</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
orchestra photo, cast list, tech & show schedule
orchestra photo and added sound for cast list, tech & show schedule on cast page
</commit_message>
<xml_diff>
--- a/howTo26/How2$ production.xlsx
+++ b/howTo26/How2$ production.xlsx
@@ -1,26 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Seagate X/RVCOprod/website/howTo26/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E1623C1-D135-8449-9926-C7FB9904348E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{012C2330-2083-1845-A900-BD12F15F9B67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-26280" yWindow="760" windowWidth="21220" windowHeight="20600" activeTab="1" xr2:uid="{E38B6315-D279-724B-88A4-0AE2C1BF2347}"/>
+    <workbookView xWindow="-26280" yWindow="760" windowWidth="21220" windowHeight="20600" xr2:uid="{E38B6315-D279-724B-88A4-0AE2C1BF2347}"/>
   </bookViews>
   <sheets>
     <sheet name="Cast" sheetId="1" r:id="rId1"/>
     <sheet name="Props" sheetId="5" r:id="rId2"/>
     <sheet name="Scenes" sheetId="2" r:id="rId3"/>
     <sheet name="Book Voice" sheetId="3" r:id="rId4"/>
+    <sheet name="Scenes playbill" sheetId="6" r:id="rId5"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId5"/>
-  </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -42,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="364">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="364">
   <si>
     <t xml:space="preserve">EMERGENCY CONTACT </t>
   </si>
@@ -1645,40 +1643,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-      <xxl21:relativeUrl r:id="rId3"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="Cast"/>
-      <sheetName val="Props"/>
-      <sheetName val="Scenes"/>
-      <sheetName val="Book Voice"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1">
-        <row r="35">
-          <cell r="C35" t="str">
-            <v xml:space="preserve">Desk with drawer </v>
-          </cell>
-        </row>
-        <row r="36">
-          <cell r="C36" t="str">
-            <v>Knitting supplies and yarn</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4511,7 +4475,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" ht="409.5" x14ac:dyDescent="0.2">
       <c r="A10" s="26" t="s">
         <v>143</v>
       </c>
@@ -4525,7 +4489,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="187" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="B11" s="27">
         <v>5</v>
       </c>
@@ -4536,7 +4500,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" ht="119" x14ac:dyDescent="0.2">
       <c r="B12" s="27">
         <v>7</v>
       </c>
@@ -4550,4 +4514,543 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC26FBFD-AFA6-DF4E-A246-4409436B2AEE}">
+  <dimension ref="A1:E44"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="4.5" style="40" customWidth="1"/>
+    <col min="2" max="2" width="5" style="40" customWidth="1"/>
+    <col min="3" max="3" width="14.5" style="37" customWidth="1"/>
+    <col min="4" max="4" width="23.5" style="39" customWidth="1"/>
+    <col min="5" max="5" width="28.1640625" style="39" customWidth="1"/>
+    <col min="6" max="16384" width="10.83203125" style="40"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" s="31" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="B1" s="33" t="s">
+        <v>118</v>
+      </c>
+      <c r="C1" s="32" t="s">
+        <v>121</v>
+      </c>
+      <c r="D1" s="32" t="s">
+        <v>117</v>
+      </c>
+      <c r="E1" s="32" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B2" s="36"/>
+    </row>
+    <row r="3" spans="1:5" ht="30" x14ac:dyDescent="0.2">
+      <c r="A3" s="35" t="s">
+        <v>103</v>
+      </c>
+      <c r="B3" s="42">
+        <v>1</v>
+      </c>
+      <c r="C3" s="43" t="s">
+        <v>122</v>
+      </c>
+      <c r="D3" s="49" t="s">
+        <v>105</v>
+      </c>
+      <c r="E3" s="39" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" s="45" customFormat="1" ht="75" x14ac:dyDescent="0.2">
+      <c r="B4" s="42">
+        <f>B3+1</f>
+        <v>2</v>
+      </c>
+      <c r="C4" s="43" t="s">
+        <v>123</v>
+      </c>
+      <c r="D4" s="47" t="s">
+        <v>159</v>
+      </c>
+      <c r="E4" s="39" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="60" x14ac:dyDescent="0.2">
+      <c r="B5" s="42">
+        <f t="shared" ref="B5:B24" si="0">B4+1</f>
+        <v>3</v>
+      </c>
+      <c r="C5" s="43" t="s">
+        <v>124</v>
+      </c>
+      <c r="D5" s="49" t="s">
+        <v>116</v>
+      </c>
+      <c r="E5" s="39" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B6" s="42">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="C6" s="43" t="s">
+        <v>107</v>
+      </c>
+      <c r="E6" s="39" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B7" s="42">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="C7" s="48" t="s">
+        <v>106</v>
+      </c>
+      <c r="E7" s="39" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="60" x14ac:dyDescent="0.2">
+      <c r="B8" s="42">
+        <v>4.2</v>
+      </c>
+      <c r="C8" s="48" t="s">
+        <v>107</v>
+      </c>
+      <c r="D8" s="47" t="s">
+        <v>180</v>
+      </c>
+      <c r="E8" s="39" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="45" x14ac:dyDescent="0.2">
+      <c r="B9" s="42">
+        <v>4.2</v>
+      </c>
+      <c r="C9" s="43" t="s">
+        <v>124</v>
+      </c>
+      <c r="D9" s="47" t="s">
+        <v>182</v>
+      </c>
+      <c r="E9" s="39" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B10" s="42">
+        <v>4.2</v>
+      </c>
+      <c r="C10" s="43"/>
+      <c r="D10" s="47" t="s">
+        <v>183</v>
+      </c>
+      <c r="E10" s="39" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B11" s="42">
+        <f>B6+1</f>
+        <v>5</v>
+      </c>
+      <c r="C11" s="43" t="s">
+        <v>132</v>
+      </c>
+      <c r="E11" s="39" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="30" x14ac:dyDescent="0.2">
+      <c r="B12" s="42">
+        <v>6.1</v>
+      </c>
+      <c r="C12" s="43" t="s">
+        <v>133</v>
+      </c>
+      <c r="D12" s="49"/>
+      <c r="E12" s="39" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B13" s="42">
+        <v>6.2</v>
+      </c>
+      <c r="C13" s="43"/>
+      <c r="D13" s="47" t="s">
+        <v>186</v>
+      </c>
+      <c r="E13" s="39" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="45" x14ac:dyDescent="0.2">
+      <c r="B14" s="42">
+        <f>B12+1</f>
+        <v>7.1</v>
+      </c>
+      <c r="C14" s="43" t="s">
+        <v>137</v>
+      </c>
+      <c r="D14" s="45"/>
+      <c r="E14" s="39" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="30" x14ac:dyDescent="0.2">
+      <c r="B15" s="42">
+        <v>7.2</v>
+      </c>
+      <c r="C15" s="43"/>
+      <c r="D15" s="47" t="s">
+        <v>190</v>
+      </c>
+      <c r="E15" s="39" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B16" s="42">
+        <v>7.2</v>
+      </c>
+      <c r="C16" s="43"/>
+      <c r="D16" s="47" t="s">
+        <v>191</v>
+      </c>
+      <c r="E16" s="39" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="30" x14ac:dyDescent="0.2">
+      <c r="B17" s="42">
+        <f>B14+1</f>
+        <v>8.1</v>
+      </c>
+      <c r="C17" s="43" t="s">
+        <v>124</v>
+      </c>
+      <c r="D17" s="47" t="s">
+        <v>138</v>
+      </c>
+      <c r="E17" s="39" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B18" s="42">
+        <f t="shared" si="0"/>
+        <v>9.1</v>
+      </c>
+      <c r="C18" s="43" t="s">
+        <v>136</v>
+      </c>
+      <c r="E18" s="39" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="30" x14ac:dyDescent="0.2">
+      <c r="B19" s="42">
+        <f t="shared" si="0"/>
+        <v>10.1</v>
+      </c>
+      <c r="C19" s="43" t="s">
+        <v>161</v>
+      </c>
+      <c r="E19" s="39" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="30" x14ac:dyDescent="0.2">
+      <c r="B20" s="42">
+        <f t="shared" si="0"/>
+        <v>11.1</v>
+      </c>
+      <c r="C20" s="43" t="s">
+        <v>139</v>
+      </c>
+      <c r="D20" s="49"/>
+      <c r="E20" s="39" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B21" s="42"/>
+      <c r="C21" s="43"/>
+      <c r="D21" s="47" t="s">
+        <v>198</v>
+      </c>
+      <c r="E21" s="39" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="45" x14ac:dyDescent="0.2">
+      <c r="B22" s="42">
+        <f>B20+1</f>
+        <v>12.1</v>
+      </c>
+      <c r="C22" s="43" t="s">
+        <v>140</v>
+      </c>
+      <c r="D22" s="51" t="s">
+        <v>200</v>
+      </c>
+      <c r="E22" s="39" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B23" s="42">
+        <f t="shared" si="0"/>
+        <v>13.1</v>
+      </c>
+      <c r="C23" s="43" t="s">
+        <v>137</v>
+      </c>
+      <c r="E23" s="39" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B24" s="42">
+        <f t="shared" si="0"/>
+        <v>14.1</v>
+      </c>
+      <c r="C24" s="43" t="s">
+        <v>141</v>
+      </c>
+      <c r="D24" s="45"/>
+      <c r="E24" s="39" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="30" x14ac:dyDescent="0.2">
+      <c r="B25" s="42">
+        <v>14.2</v>
+      </c>
+      <c r="C25" s="43"/>
+      <c r="D25" s="47" t="s">
+        <v>207</v>
+      </c>
+      <c r="E25" s="39" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B26" s="42">
+        <v>14.3</v>
+      </c>
+      <c r="C26" s="43"/>
+      <c r="D26" s="47" t="s">
+        <v>205</v>
+      </c>
+      <c r="E26" s="39" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B27" s="42">
+        <v>14.4</v>
+      </c>
+      <c r="C27" s="39"/>
+      <c r="D27" s="51" t="s">
+        <v>208</v>
+      </c>
+      <c r="E27" s="39" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="45" x14ac:dyDescent="0.2">
+      <c r="A28" s="35" t="s">
+        <v>143</v>
+      </c>
+      <c r="B28" s="42">
+        <v>1</v>
+      </c>
+      <c r="C28" s="43" t="s">
+        <v>124</v>
+      </c>
+      <c r="D28" s="56" t="s">
+        <v>112</v>
+      </c>
+      <c r="E28" s="39" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="30" x14ac:dyDescent="0.2">
+      <c r="B29" s="42">
+        <f t="shared" ref="B29:B35" si="1">B28+1</f>
+        <v>2</v>
+      </c>
+      <c r="C29" s="43" t="s">
+        <v>144</v>
+      </c>
+      <c r="D29" s="49" t="s">
+        <v>146</v>
+      </c>
+      <c r="E29" s="39" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B30" s="42">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="C30" s="43" t="s">
+        <v>145</v>
+      </c>
+      <c r="D30" s="49" t="s">
+        <v>148</v>
+      </c>
+      <c r="E30" s="39" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" s="45" customFormat="1" ht="30" x14ac:dyDescent="0.2">
+      <c r="B31" s="42">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="C31" s="43" t="s">
+        <v>147</v>
+      </c>
+      <c r="D31" s="49" t="s">
+        <v>149</v>
+      </c>
+      <c r="E31" s="39" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" s="45" customFormat="1" ht="45" x14ac:dyDescent="0.2">
+      <c r="B32" s="42">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="C32" s="43" t="s">
+        <v>150</v>
+      </c>
+      <c r="D32" s="39"/>
+      <c r="E32" s="39" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="33" spans="2:5" s="45" customFormat="1" ht="45" x14ac:dyDescent="0.2">
+      <c r="B33" s="42">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="C33" s="43" t="s">
+        <v>151</v>
+      </c>
+      <c r="D33" s="39" t="s">
+        <v>114</v>
+      </c>
+      <c r="E33" s="39" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="34" spans="2:5" ht="45" x14ac:dyDescent="0.2">
+      <c r="B34" s="42">
+        <f t="shared" si="1"/>
+        <v>7</v>
+      </c>
+      <c r="C34" s="43" t="s">
+        <v>152</v>
+      </c>
+      <c r="D34" s="49" t="s">
+        <v>155</v>
+      </c>
+      <c r="E34" s="39" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="35" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B35" s="42">
+        <f t="shared" si="1"/>
+        <v>8</v>
+      </c>
+      <c r="C35" s="43"/>
+      <c r="E35" s="39" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="36" spans="2:5" ht="45" x14ac:dyDescent="0.2">
+      <c r="B36" s="42">
+        <v>9.1</v>
+      </c>
+      <c r="C36" s="43" t="s">
+        <v>145</v>
+      </c>
+      <c r="D36" s="45"/>
+      <c r="E36" s="39" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="37" spans="2:5" ht="30" x14ac:dyDescent="0.2">
+      <c r="B37" s="42">
+        <v>9.1999999999999993</v>
+      </c>
+      <c r="C37" s="43" t="s">
+        <v>157</v>
+      </c>
+      <c r="D37" s="49" t="s">
+        <v>156</v>
+      </c>
+      <c r="E37" s="39" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="38" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B38" s="42" t="s">
+        <v>220</v>
+      </c>
+      <c r="C38" s="43"/>
+      <c r="D38" s="49"/>
+      <c r="E38" s="39" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="39" spans="2:5" ht="30" x14ac:dyDescent="0.2">
+      <c r="B39" s="42">
+        <f>B36+1</f>
+        <v>10.1</v>
+      </c>
+      <c r="C39" s="43" t="s">
+        <v>124</v>
+      </c>
+      <c r="D39" s="51" t="s">
+        <v>160</v>
+      </c>
+      <c r="E39" s="39" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="40" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B40" s="42"/>
+      <c r="C40" s="43"/>
+    </row>
+    <row r="41" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="C41" s="39"/>
+    </row>
+    <row r="42" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="C42" s="43"/>
+    </row>
+    <row r="43" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="C43" s="43"/>
+    </row>
+    <row r="44" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="C44" s="43"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
 </file>
</xml_diff>